<commit_message>
Release v1.1 - Auto Resolve before rejection summary
</commit_message>
<xml_diff>
--- a/output/DASHBOARD.xlsx
+++ b/output/DASHBOARD.xlsx
@@ -523,7 +523,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>18:58:42</t>
+          <t>10:51:15</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>133 sec</t>
+          <t>158 sec</t>
         </is>
       </c>
     </row>

</xml_diff>